<commit_message>
Audit Heritage SWIs (201, 203) against pre-conversion SWIs; restore induction and records lines; split register per series
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Register-SWI-201.xlsx
+++ b/docs/Register-SWI-201.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 201'!$A$1:$Q$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -729,7 +729,7 @@
         <v>6</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         <v>4</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         <v>5</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
         <v>6</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2729,22 +2729,22 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-201-013</t>
+          <t>SWI-PRO-MET-201-008</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Gold Elution, Electrowinning and Pre-Soak Solution Sampling</t>
+          <t>CIL Tail Sampling at Carbon Safety Screen 032-SC-003 Undersize</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Catatan</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Draft for review: Steps 3, 4 and 5 are taken from the Martabe work instructions Electrowinning Survey (DOC-3-MET-PRS-WIN-00052-IE), Elution Survey (DOC-3-MET-PRS-WIN-00053-IE) and Acid Wash Survey (DOC-3-MET-PMC-WIN-00107-IE), v1.0, 25/12/2024 and 25/01/2025. They are approved for inclusion. JSEA-PRO-MET-201-013 must be updated for the added hazards before this instruction is approved.</t>
+          <t>Safety-critical finding - read before starting. 032-SC-003 is the SOLE carbon barrier between the CIL circuit and the resin circuit. The Control Philosophy mark-up dated 07-08-2026 deletes every automatic action that closed feed valves 032-XV-003 and 032-XV-004 - item PCP-054 removes the high-level close, PCP-079 removes ILHH-041001 closing them, and PCP-122 removes the same action again from Section 3.1.7. RA-02 Rev A had already found that 032-XV-004 had no interlock. After the mark-up NEITHER valve has one. The barrier is this screen and the operator watching it. Carbon seen in the undersize is reported immediately.</t>
         </is>
       </c>
     </row>
@@ -2761,56 +2761,56 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Open items</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Open items: (1) Step 4 samples during the heating stage, which Step 2 does not allow - the JSEA must define the controls; (2) quantity and purpose of the caustic soda in the dark bottles are not stated; (3) which stage is the early stage of an electrowinning run is not stated; (4) the acid wash rinse end-point pH and acid strength are not stated; (5) confirm the HCl respirator and PPE with HSE; (6) confirm the record folders and forms exist at Mt. Morgan.</t>
+          <t>Draft for review: Steps 3, 4 and 5 are taken from the Martabe work instructions Electrowinning Survey (DOC-3-MET-PRS-WIN-00052-IE), Elution Survey (DOC-3-MET-PRS-WIN-00053-IE) and Acid Wash Survey (DOC-3-MET-PMC-WIN-00107-IE), v1.0, 25/12/2024 and 25/01/2025. They are approved for inclusion. JSEA-PRO-MET-201-013 must be updated for the added hazards before this instruction is approved.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-201-019</t>
+          <t>SWI-PRO-MET-201-013</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Water Treatment Plant Feed and Discharge Sampling</t>
+          <t>Gold Elution, Electrowinning and Pre-Soak Solution Sampling</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Catatan</t>
+          <t>Open items</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Note: the sampling points need to be updated. The points for water treatment plant No. 1 and No. 2 feed and discharge, and for the raw and filtrate water, are to be confirmed against the plant. The sampling technique in Steps 2 and 3 is taken from the Martabe work instruction Sampling Raw and Filtrat Water (DOC-3-MET-PRS-WIN-00063-IE, v1.0, 25/12/2024), where the raw water point is next to the vertical SLS ladder and the filtrate point is below it. The assay suite and the laboratory are to be set. JSEA-PRO-MET-201-019 must be updated for the added hazard.</t>
+          <t>Open items: (1) Step 4 samples during the heating stage, which Step 2 does not allow - the JSEA must define the controls; (2) quantity and purpose of the caustic soda in the dark bottles are not stated; (3) which stage is the early stage of an electrowinning run is not stated; (4) the acid wash rinse end-point pH and acid strength are not stated; (5) confirm the HCl respirator and PPE with HSE; (6) confirm the record folders and forms exist at Mt. Morgan.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-201-020</t>
+          <t>SWI-PRO-MET-201-019</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Reagent Solution Strength Sampling - NaCN, NaOH, H2SO4, NaCl, Lime and NaSH</t>
+          <t>Water Treatment Plant Feed and Discharge Sampling</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Catatan</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Draft for review: Steps 4 to 6 are taken from the Martabe work instructions Sampling Feed, Product and Final Product of Lime Slaker (DOC-3-MET-PRS-WIN-00059-IE), Sampling Hydrated Lime (DOC-3-MET-PRS-WIN-00061-IE) and ReCYN Plant Caustic Strength Measurement (DOC-3-MET-PMC-WIN-00088-IE). Step 7 is taken from Tailing Flocculant Solution Sampling (DOC-3-MET-PRS-WIN-00064-IE), moved here from the area of the tails thickener. All v1.0, 25/12/2024. JSEA-PRO-MET-201-020 must be updated for the added hazards before this instruction is approved.</t>
+          <t>Note: the sampling points need to be updated. The points for water treatment plant No. 1 and No. 2 feed and discharge, and for the raw and filtrate water, are to be confirmed against the plant. The sampling technique in Steps 2 and 3 is taken from the Martabe work instruction Sampling Raw and Filtrat Water (DOC-3-MET-PRS-WIN-00063-IE, v1.0, 25/12/2024), where the raw water point is next to the vertical SLS ladder and the filtrate point is below it. The assay suite and the laboratory are to be set. JSEA-PRO-MET-201-019 must be updated for the added hazard.</t>
         </is>
       </c>
     </row>
@@ -2827,34 +2827,34 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Open items</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Open items: (1) map the Martabe lime slaker feed hopper, product hopper and lime tank to the Transmin slaking plant points; (2) the source gives no test for the lime samples, no slurry temperature and no bag type; (3) confirm the test on hydrated lime - per cent solids on dry lime is unusual (lime availability is in SWI-PRO-MET-205-005); (4) confirm the ReCYN caustic pump drain pipe carries the diluted solution; (5) the flocculant solution strength test is not stated; (6) confirm the record folders and forms exist at Mt. Morgan.</t>
+          <t>Draft for review: Steps 4 to 6 are taken from the Martabe work instructions Sampling Feed, Product and Final Product of Lime Slaker (DOC-3-MET-PRS-WIN-00059-IE), Sampling Hydrated Lime (DOC-3-MET-PRS-WIN-00061-IE) and ReCYN Plant Caustic Strength Measurement (DOC-3-MET-PMC-WIN-00088-IE). Step 7 is taken from Tailing Flocculant Solution Sampling (DOC-3-MET-PRS-WIN-00064-IE), moved here from the area of the tails thickener. All v1.0, 25/12/2024. JSEA-PRO-MET-201-020 must be updated for the added hazards before this instruction is approved.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-201-022</t>
+          <t>SWI-PRO-MET-201-020</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Online Analyser Verification Sampling - pH, Cyanide and Dissolved Oxygen</t>
+          <t>Reagent Solution Strength Sampling - NaCN, NaOH, H2SO4, NaCl, Lime and NaSH</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Open items</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Draft for review: Steps 4 and 5 are taken from the Martabe work instructions Verifikasi Analyzer Leaching (12/05/2025) and Check pH Tailing Slurry Solution (DOC-3-MET-PMC-WIN-00106-IE, 25/01/2025). JSEA-PRO-MET-201-022 must be updated for the added hazards before this instruction is approved.</t>
+          <t>Open items: (1) map the Martabe lime slaker feed hopper, product hopper and lime tank to the Transmin slaking plant points; (2) the source gives no test for the lime samples, no slurry temperature and no bag type; (3) confirm the test on hydrated lime - per cent solids on dry lime is unusual (lime availability is in SWI-PRO-MET-205-005); (4) confirm the ReCYN caustic pump drain pipe carries the diluted solution; (5) the flocculant solution strength test is not stated; (6) confirm the record folders and forms exist at Mt. Morgan.</t>
         </is>
       </c>
     </row>
@@ -2871,17 +2871,39 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review: Steps 4 and 5 are taken from the Martabe work instructions Verifikasi Analyzer Leaching (12/05/2025) and Check pH Tailing Slurry Solution (DOC-3-MET-PMC-WIN-00106-IE, 25/01/2025). JSEA-PRO-MET-201-022 must be updated for the added hazards before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-201-022</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Online Analyser Verification Sampling - pH, Cyanide and Dissolved Oxygen</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
           <t>Open items</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Open items: (1) the quantity of caustic or the target pH is not stated in the source - hold the solution above pH 10.5 in line with the HCN controls; (2) the tolerance for the pH probe check is only given by an example of about 0.2 pH, which must not erode the cyanide safety margin of pH 10.5; (3) the source uses buffers 7 and 10 only, whereas SWI-PRO-MET-206-004 uses 4, 7 and 10 - confirm the buffers cover the working range of the probe; (4) the tolerance per loop is to be set; (5) confirm the record folders exist at Mt. Morgan.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2901,21 +2923,21 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Register seri 201 Plant Sampling, SWI-PRO-MET-201-001 sampai 201-025 (25 dokumen).</t>
+          <t>Register seri 201 Plant Sampling (25 dokumen dalam format Heritage).</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Semua dokumen sudah dalam format Heritage. Data dibaca langsung dari Part 1 dan Part 2 tiap dokumen (judul, tanggal, owner, JSEA ID, area, frekuensi).</t>
+          <t>Data dibaca langsung dari Part 1 dan Part 2 tiap dokumen (judul, tanggal, owner, JSEA ID, area, frekuensi).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Klasifikasi dan padanan Martabe diambil dari docs/Matriks-Rujukan-Martabe.xlsx dan docs/Tabel-SWI-vs-Martabe.xlsx. Format Heritage tidak memuat kolom klasifikasi, jadi klasifikasi hanya ada di register.</t>
+          <t>Klasifikasi dan padanan Martabe diambil dari docs/Matriks-Rujukan-Martabe.xlsx dan docs/Tabel-SWI-vs-Martabe.xlsx, ditimpa oleh keputusan review bila ada. Format Heritage tidak memuat kolom klasifikasi, jadi klasifikasi hanya ada di register.</t>
         </is>
       </c>
     </row>
@@ -2929,14 +2951,14 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Status isi: Final = tanpa tambahan Martabe; DRAFT FOR REVIEW = ada tambahan Martabe yang belum disetujui JSEA; Catatan = ada catatan yang perlu ditindaklanjuti.</t>
+          <t>Status isi: Final = tanpa tambahan Martabe terbuka; DRAFT FOR REVIEW = ada tambahan Martabe yang menunggu JSEA; Catatan = ada catatan yang perlu ditindaklanjuti.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Sheet "Draft dan open items" memuat semua paragraf draft, catatan, dan open items yang tercatat di Description of work.</t>
+          <t>Sheet "Draft dan open items" memuat paragraf draft, catatan, temuan safety-critical, dan open items di Description of work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove parent-procedure and register statements from all SWIs and SWPs; drop MM-4034-033-OR-03- prefix from file names
- SWI: delete the 'This instruction sits under Standard Work Procedure ...' and
  'Register line: ...' statements, and the parent procedure and SWI/SWMS register
  rows of the Referenced Documents table.
- SWP: delete the register-area sentence and bullet, the register file paragraph
  and the register-tab sentence; Register Traceability becomes Document Traceability.
- Rename SWI and SWP files to start with SWI- / SWP-; registers updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Register-SWI-201.xlsx
+++ b/docs/Register-SWI-201.xlsx
@@ -665,7 +665,7 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-001-Front-End-Sampling-Round---Scrubber-Discharge-Hopper-and-Trash-Scr-RevA.docx</t>
+          <t>SWI-PRO-MET-201-001-Front-End-Sampling-Round---Scrubber-Discharge-Hopper-and-Trash-Scr-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
         <v>6</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-002-IsaMill-Feed-and-Discharge-Sampling-Round-RevA.docx</t>
+          <t>SWI-PRO-MET-201-002-IsaMill-Feed-and-Discharge-Sampling-Round-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
         <v>7</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-003-Leach-Tank-Sampling-Round---031-TK-001-Launder-and-Discharge-RevA.docx</t>
+          <t>SWI-PRO-MET-201-003-Leach-Tank-Sampling-Round---031-TK-001-Launder-and-Discharge-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-004-CIL-Sampling-Round---032-TK-002-to-032-TK-006-Launders-RevA.docx</t>
+          <t>SWI-PRO-MET-201-004-CIL-Sampling-Round---032-TK-002-to-032-TK-006-Launders-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
         <v>4</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
@@ -997,7 +997,7 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-005-Carbon-Concentration-Measurement-in-CIL-Tanks-RevA.docx</t>
+          <t>SWI-PRO-MET-201-005-Carbon-Concentration-Measurement-in-CIL-Tanks-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-006-Loaded-Carbon-Sampling-at-Loaded-Carbon-Screen-032-SC-002-RevA.docx</t>
+          <t>SWI-PRO-MET-201-006-Loaded-Carbon-Sampling-at-Loaded-Carbon-Screen-032-SC-002-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-007-Barren-Carbon-Sampling-at-Carbon-Dewatering-Screen-061-SC-013-RevA.docx</t>
+          <t>SWI-PRO-MET-201-007-Barren-Carbon-Sampling-at-Carbon-Dewatering-Screen-061-SC-013-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1227,7 @@
         <v>5</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-008-CIL-Tail-Sampling-at-Carbon-Safety-Screen-032-SC-003-Undersize-RevA.docx</t>
+          <t>SWI-PRO-MET-201-008-CIL-Tail-Sampling-at-Carbon-Safety-Screen-032-SC-003-Undersize-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-009-Metal-Adsorption-Sampling-Round---041-TK-007-and-041-TK-008-ReCYN-RevA.docx</t>
+          <t>SWI-PRO-MET-201-009-Metal-Adsorption-Sampling-Round---041-TK-007-and-041-TK-008-ReCYN-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-010-Cyanide-Adsorption-Sampling-Round---051-TK-009-and-051-TK-010-ReCY-RevA.docx</t>
+          <t>SWI-PRO-MET-201-010-Cyanide-Adsorption-Sampling-Round---051-TK-009-and-051-TK-010-ReCY-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
         <v>4</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-011-Resin-Concentration-Measurement-in-Adsorption-Tanks-RevA.docx</t>
+          <t>SWI-PRO-MET-201-011-Resin-Concentration-Measurement-in-Adsorption-Tanks-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-012-Loaded-and-Barren-Resin-Sampling-at-Screens-and-Hoppers-RevA.docx</t>
+          <t>SWI-PRO-MET-201-012-Loaded-and-Barren-Resin-Sampling-at-Screens-and-Hoppers-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
         <v>6</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-013-Gold-Elution-Electrowinning-and-Pre-Soak-Solution-Sampling-RevA.docx</t>
+          <t>SWI-PRO-MET-201-013-Gold-Elution-Electrowinning-and-Pre-Soak-Solution-Sampling-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-014-Copper-Elution-Reactor-and-Thickener-Sampling-RevA.docx</t>
+          <t>SWI-PRO-MET-201-014-Copper-Elution-Reactor-and-Thickener-Sampling-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-015-Copper-Filtrate-and-Precipitate-Sampling-RevA.docx</t>
+          <t>SWI-PRO-MET-201-015-Copper-Filtrate-and-Precipitate-Sampling-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-016-Cyanide-Elution-Stripping-and-AVR-Sampling-RevA.docx</t>
+          <t>SWI-PRO-MET-201-016-Cyanide-Elution-Stripping-and-AVR-Sampling-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-017-Tails-Thickener-Feed-Overflow-and-Underflow-Sampling-RevA.docx</t>
+          <t>SWI-PRO-MET-201-017-Tails-Thickener-Feed-Overflow-and-Underflow-Sampling-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-018-Final-Tailings-and-TSF-Return-Water-Sampling-RevA.docx</t>
+          <t>SWI-PRO-MET-201-018-Final-Tailings-and-TSF-Return-Water-Sampling-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
         <v>5</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-019-Water-Treatment-Plant-Feed-and-Discharge-Sampling-RevA.docx</t>
+          <t>SWI-PRO-MET-201-019-Water-Treatment-Plant-Feed-and-Discharge-Sampling-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-020-Reagent-Solution-Strength-Sampling---NaCN-NaOH-H2SO4-NaCl-Lime-and-RevA.docx</t>
+          <t>SWI-PRO-MET-201-020-Reagent-Solution-Strength-Sampling---NaCN-NaOH-H2SO4-NaCl-Lime-and-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-021-Composite-Sample-Build-Up-Splitting-and-Handover-to-Laboratory-RevA.docx</t>
+          <t>SWI-PRO-MET-201-021-Composite-Sample-Build-Up-Splitting-and-Handover-to-Laboratory-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-022-Online-Analyser-Verification-Sampling---pH-Cyanide-and-Dissolved-O-RevA.docx</t>
+          <t>SWI-PRO-MET-201-022-Online-Analyser-Verification-Sampling---pH-Cyanide-and-Dissolved-O-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-023-Sample-Point-Access-Isolation-Flushing-and-Housekeeping-RevA.docx</t>
+          <t>SWI-PRO-MET-201-023-Sample-Point-Access-Isolation-Flushing-and-Housekeeping-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-024-Sampling-During-Start-Up-Shutdown-and-Upset-Conditions-RevA.docx</t>
+          <t>SWI-PRO-MET-201-024-Sampling-During-Start-Up-Shutdown-and-Upset-Conditions-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-201-025-Sampling-Under-Cyanide-Alarm-or-Restricted-Access-Conditions-RevA.docx</t>
+          <t>SWI-PRO-MET-201-025-Sampling-Under-Cyanide-Alarm-or-Restricted-Access-Conditions-RevA.docx</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -2962,13 +2962,6 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Referensi register: HM-MMM-WHS-REG-XXX-R00-SWI-SWMS, tab SWI-MET.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>